<commit_message>
finished ish solar panel excel
</commit_message>
<xml_diff>
--- a/PowerBudgeting/PowerBudgeting.xlsx
+++ b/PowerBudgeting/PowerBudgeting.xlsx
@@ -8,36 +8,135 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Main Engineering\Engineering\Project Genesis EE Notes\PowerBudgeting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7CF2652-4991-4D8C-AD06-89B685E9D7A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BFFC162-1FD0-4E97-84FE-F970C19B8B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Main" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
-  <si>
-    <t>test</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+  <si>
+    <t>Battery Cells</t>
+  </si>
+  <si>
+    <t>Molicel P30B 18650</t>
+  </si>
+  <si>
+    <t>Capacity (wH)</t>
+  </si>
+  <si>
+    <t>Worst</t>
+  </si>
+  <si>
+    <t>Typical</t>
+  </si>
+  <si>
+    <t>Solar Panels</t>
+  </si>
+  <si>
+    <t>Efficiency (%)</t>
+  </si>
+  <si>
+    <t>Solar Irradiance (W/m^2)</t>
+  </si>
+  <si>
+    <t>Area Facing Sun (m^2)</t>
+  </si>
+  <si>
+    <t>Pointing Accuracy (±deg)</t>
+  </si>
+  <si>
+    <t>Power Generation in Sunlight (W)</t>
+  </si>
+  <si>
+    <t>Orbits Per Day</t>
+  </si>
+  <si>
+    <t>Orbit Period (min)</t>
+  </si>
+  <si>
+    <t>Beta_Critical (deg)</t>
+  </si>
+  <si>
+    <t>Radius of Earth (km)</t>
+  </si>
+  <si>
+    <t>height (km)</t>
+  </si>
+  <si>
+    <t>Eclipse Period (min)</t>
+  </si>
+  <si>
+    <t>Sunlight Period (min)</t>
+  </si>
+  <si>
+    <t>Net Generation in Sunlight (W)</t>
+  </si>
+  <si>
+    <t>Quiescent Load Power (W)</t>
+  </si>
+  <si>
+    <t>Net Energy Generated Per Orbit (Wh)</t>
+  </si>
+  <si>
+    <t>Time to Fully Charge Battery (hr)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -51,7 +150,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -59,14 +158,59 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -345,15 +489,232 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B4"/>
+  <dimension ref="B3:G36"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B3" s="4" t="s">
         <v>0</v>
       </c>
+      <c r="C3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="G3" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B4" s="4"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="2">
+        <f>C8*D8*B14*MAX(0, COS(RADIANS(B11)))</f>
+        <v>2.5578433137792427</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B5" s="4"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="2">
+        <v>10.4</v>
+      </c>
+      <c r="E5" s="2">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="G6" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B7" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="2">
+        <f>G4-D11</f>
+        <v>1.5578433137792427</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B8" s="4"/>
+      <c r="C8" s="3">
+        <f>20/100</f>
+        <v>0.2</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="G9" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B10" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="2">
+        <f>G7*(B35/60)</f>
+        <v>1.2601228502736872</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B11" s="2">
+        <v>20</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="G12" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B13" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="2">
+        <f>((E5/G10)*B20)/60</f>
+        <v>13.712948698808963</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B14" s="2">
+        <v>1361</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B16" s="7" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B17" s="2">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B18" s="1"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B19" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B20" s="2">
+        <f>(24*60)/B17</f>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B21" s="1"/>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B22" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B23" s="3">
+        <v>6378</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B25" s="7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B26" s="2">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B27" s="1"/>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B28" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B29" s="2">
+        <f>DEGREES(ASIN(B23/(B23+B26)))</f>
+        <v>68.018452171858542</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B30" s="1"/>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B31" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B32" s="2">
+        <f>(B20/PI())*ACOS(RADIANS((SQRT((B23+B26)^2-B23^2))/((B23+B26)*COS(RADIANS(B29)))))</f>
+        <v>47.466639585850338</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B33" s="1"/>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B34" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B35" s="2">
+        <f>B20-B32</f>
+        <v>48.533360414149662</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B36" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="B3:B5"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="B7:B8"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C3:C5" r:id="rId1" display="Molicel P30B 18650" xr:uid="{EB2EE773-CD21-4599-BA06-953E50EF070E}"/>
+    <hyperlink ref="B13" r:id="rId2" xr:uid="{6A7A2EBC-F41C-4C55-B861-E94BB1EEB00E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>